<commit_message>
[20 23] update excel_zad2 number format
</commit_message>
<xml_diff>
--- a/day_20_31_08_2025/xlsxwriter3.xlsx
+++ b/day_20_31_08_2025/xlsxwriter3.xlsx
@@ -29,8 +29,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy/mm/dd"/>
+    <numFmt numFmtId="165" formatCode="[$-409]0.00"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -90,12 +91,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -390,7 +392,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:1">
@@ -413,6 +415,11 @@
         <v>42656</v>
       </c>
     </row>
+    <row r="5" spans="1:1">
+      <c r="A5" s="3">
+        <v>3.3333333</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>